<commit_message>
update new UI and workflow
</commit_message>
<xml_diff>
--- a/data/budget.xlsx
+++ b/data/budget.xlsx
@@ -3,49 +3,38 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17920"/>
+  </bookViews>
   <sheets>
     <sheet sheetId="1" name="Projects" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Transactions" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="60">
   <si>
     <t>id</t>
   </si>
   <si>
+    <t>no</t>
+  </si>
+  <si>
     <t>projectCode</t>
   </si>
   <si>
     <t>projectName</t>
   </si>
   <si>
-    <t>department</t>
-  </si>
-  <si>
-    <t>budgetCategory</t>
+    <t>category</t>
   </si>
   <si>
     <t>owner</t>
   </si>
   <si>
-    <t>budgetAmount</t>
-  </si>
-  <si>
-    <t>spentAmount</t>
-  </si>
-  <si>
-    <t>balanceAmount</t>
-  </si>
-  <si>
-    <t>status</t>
-  </si>
-  <si>
-    <t>priority</t>
-  </si>
-  <si>
     <t>startDate</t>
   </si>
   <si>
@@ -55,10 +44,164 @@
     <t>remark</t>
   </si>
   <si>
+    <t>logoPath</t>
+  </si>
+  <si>
     <t>createdAt</t>
   </si>
   <si>
     <t>updatedAt</t>
+  </si>
+  <si>
+    <t>2cae81ea-e9ab-44bb-96cb-a6d346f17666</t>
+  </si>
+  <si>
+    <t>GB-00001</t>
+  </si>
+  <si>
+    <t>Glori Creativity Sole Co.,Ltd</t>
+  </si>
+  <si>
+    <t>Administrative expenses</t>
+  </si>
+  <si>
+    <t>Glori</t>
+  </si>
+  <si>
+    <t>2026-01-01</t>
+  </si>
+  <si>
+    <t>2026-12-31</t>
+  </si>
+  <si>
+    <t>/uploads/1773740621694-Company-name.png</t>
+  </si>
+  <si>
+    <t>2026-03-17T09:43:41.725Z</t>
+  </si>
+  <si>
+    <t>2026-03-17T09:57:30.142Z</t>
+  </si>
+  <si>
+    <t>1888d0ca-e6a6-447a-aa35-3dc3bbaf8757</t>
+  </si>
+  <si>
+    <t>GB-00002</t>
+  </si>
+  <si>
+    <t>Exploration Mining</t>
+  </si>
+  <si>
+    <t>Bag, Document envelope</t>
+  </si>
+  <si>
+    <t>Toto</t>
+  </si>
+  <si>
+    <t>2026-03-17</t>
+  </si>
+  <si>
+    <t>2026-04-17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Product Name: Document envelope
+Size: A4
+Material: Paper
+Logo: 1 Position
+Product Name: Bags
+Size: 35×25×12 cm
+Material: canvar A12
+Logo: 2 Position</t>
+  </si>
+  <si>
+    <t>/uploads/1773740916417-PHOTO-2026-03-11-17-01-02_2.jpg</t>
+  </si>
+  <si>
+    <t>2026-03-17T09:48:36.429Z</t>
+  </si>
+  <si>
+    <t>projectId</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>currency</t>
+  </si>
+  <si>
+    <t>amount</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>billPath</t>
+  </si>
+  <si>
+    <t>b7f7a8db-3e29-4fad-a676-69424a58b235</t>
+  </si>
+  <si>
+    <t>expense</t>
+  </si>
+  <si>
+    <t>Rider</t>
+  </si>
+  <si>
+    <t>LAK</t>
+  </si>
+  <si>
+    <t>/uploads/1773740650605-WhatsApp_Image_2026-03-17_at_4_07_46_PM.jpeg</t>
+  </si>
+  <si>
+    <t>2026-03-17T09:44:10.620Z</t>
+  </si>
+  <si>
+    <t>e012b4dc-bd9b-4ca9-8210-0aa8c3c09c0f</t>
+  </si>
+  <si>
+    <t>income</t>
+  </si>
+  <si>
+    <t>Deposit</t>
+  </si>
+  <si>
+    <t>Deposit 30%</t>
+  </si>
+  <si>
+    <t>/uploads/1773741023127-PHOTO-2026-03-17-13-29-24.jpg</t>
+  </si>
+  <si>
+    <t>2026-03-17T09:50:23.144Z</t>
+  </si>
+  <si>
+    <t>5fc0587b-47b0-4506-9696-fb30c9f667c0</t>
+  </si>
+  <si>
+    <t>Facebook Ad</t>
+  </si>
+  <si>
+    <t>/uploads/1773741352134-Screenshot_2026-03-17_at_4_51_03___PM.png</t>
+  </si>
+  <si>
+    <t>2026-03-17T09:55:52.150Z</t>
+  </si>
+  <si>
+    <t>a46ec348-d002-4744-9c6d-23a312abb531</t>
+  </si>
+  <si>
+    <t>Logistic</t>
+  </si>
+  <si>
+    <t>2026-03-18</t>
+  </si>
+  <si>
+    <t>/uploads/1773814306098-WhatsApp_Image_2026-03-18_at_1_11_24_PM.jpeg</t>
+  </si>
+  <si>
+    <t>2026-03-18T06:11:46.120Z</t>
   </si>
 </sst>
 </file>
@@ -447,22 +590,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P1"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <dimension ref="A1:L3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="28" customWidth="1"/>
-    <col min="4" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="10" width="14" customWidth="1"/>
-    <col min="11" max="11" width="12" customWidth="1"/>
-    <col min="12" max="13" width="14" customWidth="1"/>
-    <col min="14" max="14" width="34" customWidth="1"/>
-    <col min="15" max="16" width="24" customWidth="1"/>
+    <col min="1" max="12" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="22" customHeight="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -499,17 +633,285 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="D2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="E2" t="s">
         <v>15</v>
+      </c>
+      <c r="F2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I3" t="s">
+        <v>29</v>
+      </c>
+      <c r="J3" t="s">
+        <v>30</v>
+      </c>
+      <c r="K3" t="s">
+        <v>31</v>
+      </c>
+      <c r="L3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:L5"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
+  <cols>
+    <col min="1" max="12" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" t="s">
+        <v>41</v>
+      </c>
+      <c r="G2" t="s">
+        <v>42</v>
+      </c>
+      <c r="H2">
+        <v>60000</v>
+      </c>
+      <c r="I2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J2" t="s">
+        <v>43</v>
+      </c>
+      <c r="K2" t="s">
+        <v>44</v>
+      </c>
+      <c r="L2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E3" t="s">
+        <v>47</v>
+      </c>
+      <c r="F3" t="s">
+        <v>48</v>
+      </c>
+      <c r="G3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H3">
+        <v>5100000</v>
+      </c>
+      <c r="I3" t="s">
+        <v>27</v>
+      </c>
+      <c r="J3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
+        <v>40</v>
+      </c>
+      <c r="E4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G4" t="s">
+        <v>42</v>
+      </c>
+      <c r="H4">
+        <v>983000</v>
+      </c>
+      <c r="I4" t="s">
+        <v>27</v>
+      </c>
+      <c r="J4" t="s">
+        <v>53</v>
+      </c>
+      <c r="K4" t="s">
+        <v>54</v>
+      </c>
+      <c r="L4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>55</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" t="s">
+        <v>40</v>
+      </c>
+      <c r="E5" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" t="s">
+        <v>56</v>
+      </c>
+      <c r="G5" t="s">
+        <v>42</v>
+      </c>
+      <c r="H5">
+        <v>34000</v>
+      </c>
+      <c r="I5" t="s">
+        <v>57</v>
+      </c>
+      <c r="J5" t="s">
+        <v>58</v>
+      </c>
+      <c r="K5" t="s">
+        <v>59</v>
+      </c>
+      <c r="L5" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update budget excel file
</commit_message>
<xml_diff>
--- a/data/budget.xlsx
+++ b/data/budget.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11008"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02095C5B-BCCC-5541-81E7-6D6FC3EC8B76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17920"/>
+    <workbookView xWindow="-38400" yWindow="-1360" windowWidth="38400" windowHeight="21000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Projects" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Transactions" state="visible" r:id="rId5"/>
+    <sheet name="Projects" sheetId="1" r:id="rId1"/>
+    <sheet name="Transactions" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="248">
   <si>
     <t>id</t>
   </si>
@@ -104,7 +105,7 @@
     <t>2026-04-17</t>
   </si>
   <si>
-    <t xml:space="preserve">Product Name: Document envelope
+    <t>Product Name: Document envelope
 Size: A4
 Material: Paper
 Logo: 1 Position
@@ -203,22 +204,667 @@
   <si>
     <t>2026-03-18T06:11:46.120Z</t>
   </si>
+  <si>
+    <t>0b79e4a5-5a10-48f1-acef-11f7a7b6cd5d</t>
+  </si>
+  <si>
+    <t>GB-00003</t>
+  </si>
+  <si>
+    <t>tourism Malaysia in Vientiane</t>
+  </si>
+  <si>
+    <t>Bag, Notebook</t>
+  </si>
+  <si>
+    <t>Bin</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>2026-04-13</t>
+  </si>
+  <si>
+    <t>Product Name: Bags
+Size: 30*43*20cm
+Material: Linen fabric
+Logo: 2 Position
+Product Name: Noted
+Book
+Size: 30*43*20cm
+Material: Paper
+Logo: 2 Position</t>
+  </si>
+  <si>
+    <t>/uploads/1773913004907-WhatsApp_Image_2026-03-18_at_6_06_21___PM.jpeg</t>
+  </si>
+  <si>
+    <t>2026-03-19T09:36:45.433Z</t>
+  </si>
+  <si>
+    <t>07b5482a-fdaf-4c83-9d00-0c7bb6de9063</t>
+  </si>
+  <si>
+    <t>GB-00004</t>
+  </si>
+  <si>
+    <t>HYUNDAI</t>
+  </si>
+  <si>
+    <t>Car Front Windshield Sunshade</t>
+  </si>
+  <si>
+    <t>Product Name: Car Front
+Windshield Sunshade
+Size: 140×126×80 cm
+Material: Titanium Silver,
+Large: 372g
+Logo: 3 Position
+Remark: Start 2000 pcs
+Product Name: Car Front
+Windshield Sunshade
+Size: 140×126×80 cm
+Material: Titanium Silver,
+Large: 372g
+Logo: 3 Position
+Remark: Start 2000 pcs
+Product Name: Car Front
+Windshield Sunshade
+Size: 140×126×80 cm
+Material: Titanium Silver,
+Large: 372g
+Logo: 3 Position
+Remark: Start 2000 pcs
+Color of Car Front
+Windshield Sunshade and
+handle
+Color of Car Front
+Windshield Sunshade and
+handle
+Color of Bags</t>
+  </si>
+  <si>
+    <t>/uploads/1773915863014-PHOTO-2026-03-19-17-22-27.jpg</t>
+  </si>
+  <si>
+    <t>2026-03-19T10:24:23.179Z</t>
+  </si>
+  <si>
+    <t>8a006c37-9aa5-4544-9f44-8d8f5f531b5c</t>
+  </si>
+  <si>
+    <t>GB-00005</t>
+  </si>
+  <si>
+    <t>TMNPB</t>
+  </si>
+  <si>
+    <t>coffee cup plate set, shoes</t>
+  </si>
+  <si>
+    <t>2026-04-21</t>
+  </si>
+  <si>
+    <t>Product Name: Caps and dish
+Size: 350 ml
+Material: ceramic
+Logo: 2 Position
+Product Name: Caps
+Size: 380 ml
+Material: ceramic
+Logo: 1 PositionProduct Name: shoes
+Size: 23 ml
+Material: Plastic
+Logo: 1 Position</t>
+  </si>
+  <si>
+    <t>/uploads/1774610163459-PHOTO-2026-03-27-16-48-13.jpg</t>
+  </si>
+  <si>
+    <t>2026-03-27T11:16:04.805Z</t>
+  </si>
+  <si>
+    <t>003473d8-e840-42ad-9465-0fe5c7244715</t>
+  </si>
+  <si>
+    <t>GB-00006</t>
+  </si>
+  <si>
+    <t>TOYOTA Lao Service</t>
+  </si>
+  <si>
+    <t>Shirt, Bottle, Umbrella, Pillow, cap</t>
+  </si>
+  <si>
+    <t>2026-05-01</t>
+  </si>
+  <si>
+    <t>Product Name: Polo shirt
+Capacity: 550ml
+Material: Stainless Steel 304, art
+Logo: 1 Position
+Product Name: Bottle
+Capacity: 550ml
+Material: Stainless Steel 304
+Logo: 1 Position
+Product Name: Umbrella (UV
+Coating), Automatic close
+Size: 21inches
+Ribs: 8 ribs
+Logo: 4 positions, full color printing
+Product Name: Umberalla (UV
+Coating), Automatic close
+Size: 21inches
+Ribs: 8 ribs
+Logo: 4 positions, full color
+printing
+Product Name: Umbrella Doublelayer
+size: 30 inch
+Material: fiber glass , save UV
+Logo: 4 Position
+Product Name: Car neck pillow
+Material: fabric
+Size : 19*26 cm
+printing: logo 1 point
+Product Name: caps
+Material: cotton
+Size : 54-62
+printing: logo 1 point</t>
+  </si>
+  <si>
+    <t>/uploads/1775455056621-toyota-brand-logo-car-symbol-with-name-black-design-japan-automobile-illustratio.jpg</t>
+  </si>
+  <si>
+    <t>2026-04-06T05:57:36.623Z</t>
+  </si>
+  <si>
+    <t>3cf7944d-d78a-4c58-846a-8c69fa6f2f5e</t>
+  </si>
+  <si>
+    <t>GB-00007</t>
+  </si>
+  <si>
+    <t>MAISONNONGKHIAW</t>
+  </si>
+  <si>
+    <t>Mug</t>
+  </si>
+  <si>
+    <t>Name: Mug
+Material: ceramic
+size: 350ml
+logo: 2 point</t>
+  </si>
+  <si>
+    <t>/uploads/1775455299324-Unknown</t>
+  </si>
+  <si>
+    <t>2026-04-06T06:01:39.326Z</t>
+  </si>
+  <si>
+    <t>f1ddfec2-88e5-4cdb-b770-f9ff11895423</t>
+  </si>
+  <si>
+    <t>Logistics rider</t>
+  </si>
+  <si>
+    <t>2026-03-19</t>
+  </si>
+  <si>
+    <t>/uploads/1773913867243-PHOTO-2026-03-19-16-37-39.jpg</t>
+  </si>
+  <si>
+    <t>2026-03-19T09:51:08.376Z</t>
+  </si>
+  <si>
+    <t>f986bf96-d234-4273-a864-523442756a69</t>
+  </si>
+  <si>
+    <t>investment</t>
+  </si>
+  <si>
+    <t>Order production</t>
+  </si>
+  <si>
+    <t>Bag</t>
+  </si>
+  <si>
+    <t>/uploads/1773914342487-PHOTO-2026-03-19-16-52-03.jpg</t>
+  </si>
+  <si>
+    <t>2026-03-19T09:59:02.653Z</t>
+  </si>
+  <si>
+    <t>1d60ae76-81fa-468c-8019-98d4dee10571</t>
+  </si>
+  <si>
+    <t>/uploads/1773914598263-PHOTO-2026-03-19-16-59-55.jpg</t>
+  </si>
+  <si>
+    <t>2026-03-19T10:03:18.428Z</t>
+  </si>
+  <si>
+    <t>813a8786-a22d-4b95-b749-4c8702f13ccc</t>
+  </si>
+  <si>
+    <t>Example</t>
+  </si>
+  <si>
+    <t>/uploads/1773915970126-PHOTO-2026-03-19-17-11-45.jpg</t>
+  </si>
+  <si>
+    <t>2026-03-19T10:26:10.843Z</t>
+  </si>
+  <si>
+    <t>44d19cd2-c289-41cb-9738-19d79fed5611</t>
+  </si>
+  <si>
+    <t>Document envelopes</t>
+  </si>
+  <si>
+    <t>/uploads/1773916100909-PHOTO-2026-03-19-17-02-52.jpg</t>
+  </si>
+  <si>
+    <t>2026-03-19T10:28:21.074Z</t>
+  </si>
+  <si>
+    <t>b4bc11a6-58af-4bc1-8258-96b3fd283cc6</t>
+  </si>
+  <si>
+    <t>2026-03-20</t>
+  </si>
+  <si>
+    <t>/uploads/1773983644645-PHOTO-2026-03-19-18-42-47.jpg</t>
+  </si>
+  <si>
+    <t>2026-03-20T05:14:05.995Z</t>
+  </si>
+  <si>
+    <t>0d386f02-281b-49c0-a398-8191bf48b78e</t>
+  </si>
+  <si>
+    <t>Notebook</t>
+  </si>
+  <si>
+    <t>/uploads/1773984119356-WhatsApp_Image_2026-03-19_at_6_43_03___PM.jpeg</t>
+  </si>
+  <si>
+    <t>2026-03-20T05:21:59.852Z</t>
+  </si>
+  <si>
+    <t>7491ae59-b4a6-4c12-a91a-c14e5d62d175</t>
+  </si>
+  <si>
+    <t>/uploads/1773984165406-WhatsApp_Image_2026-03-19_at_6_43_03___PM__1_.jpeg</t>
+  </si>
+  <si>
+    <t>2026-03-20T05:22:45.901Z</t>
+  </si>
+  <si>
+    <t>c29ed229-9544-4ca6-9a3e-b9cf7cdaa024</t>
+  </si>
+  <si>
+    <t>Tumbler</t>
+  </si>
+  <si>
+    <t>/uploads/1773999468681-PHOTO-2026-03-20-12-36-54.jpg</t>
+  </si>
+  <si>
+    <t>2026-03-20T09:37:49.004Z</t>
+  </si>
+  <si>
+    <t>4e8b4704-7931-4f91-afbb-608b52e906b9</t>
+  </si>
+  <si>
+    <t>RAILWAY Domain (5 USD)</t>
+  </si>
+  <si>
+    <t>2026-03-21</t>
+  </si>
+  <si>
+    <t>/uploads/1774070989723-PHOTO-2026-03-21-12-23-07.jpg</t>
+  </si>
+  <si>
+    <t>2026-03-21T05:29:49.923Z</t>
+  </si>
+  <si>
+    <t>8f7c082c-7a79-4ab3-91b3-88caf9e659d1</t>
+  </si>
+  <si>
+    <t>2026-03-22</t>
+  </si>
+  <si>
+    <t>/uploads/1774177296982-PHOTO-2026-03-22-17-53-16.jpg</t>
+  </si>
+  <si>
+    <t>2026-03-22T11:01:37.147Z</t>
+  </si>
+  <si>
+    <t>e719b535-f7f1-49ca-a816-7c1b9ea4720a</t>
+  </si>
+  <si>
+    <t>Advertising services</t>
+  </si>
+  <si>
+    <t>2026-03-23</t>
+  </si>
+  <si>
+    <t>/uploads/1774243997496-PHOTO-2026-03-23-09-57-16.jpg</t>
+  </si>
+  <si>
+    <t>2026-03-23T05:33:18.054Z</t>
+  </si>
+  <si>
+    <t>bbe9e536-d049-417a-ab38-5d78ef4426e4</t>
+  </si>
+  <si>
+    <t>2026-03-24</t>
+  </si>
+  <si>
+    <t>/uploads/1774349984640-PHOTO-2026-03-24-13-09-12.jpg</t>
+  </si>
+  <si>
+    <t>2026-03-24T10:59:44.974Z</t>
+  </si>
+  <si>
+    <t>cfad3f06-9806-4981-b294-f3bb40684f04</t>
+  </si>
+  <si>
+    <t>Beach flag</t>
+  </si>
+  <si>
+    <t>2026-03-27</t>
+  </si>
+  <si>
+    <t>/uploads/1774606446959-PHOTO-2026-03-27-16-37-37.jpg</t>
+  </si>
+  <si>
+    <t>2026-03-27T10:14:07.054Z</t>
+  </si>
+  <si>
+    <t>a9a27e7e-9b88-40d8-b7f2-dc21e499dc80</t>
+  </si>
+  <si>
+    <t>/uploads/1774610513972-PHOTO-2026-03-27-16-49-15.jpg</t>
+  </si>
+  <si>
+    <t>2026-03-27T11:21:55.818Z</t>
+  </si>
+  <si>
+    <t>f72dc222-3624-48a2-825b-1784dc77b3b3</t>
+  </si>
+  <si>
+    <t>Coffee cup 30%</t>
+  </si>
+  <si>
+    <t>/uploads/1774610823238-PHOTO-2026-03-27-16-47-15.jpg</t>
+  </si>
+  <si>
+    <t>2026-03-27T11:27:04.254Z</t>
+  </si>
+  <si>
+    <t>021f56a8-2574-4f9b-abf3-49b53ff5d017</t>
+  </si>
+  <si>
+    <t>shoes 30%</t>
+  </si>
+  <si>
+    <t>/uploads/1774611053965-PHOTO-2026-03-27-16-50-06.jpg</t>
+  </si>
+  <si>
+    <t>2026-03-27T11:30:54.846Z</t>
+  </si>
+  <si>
+    <t>2cd45e7f-49c3-4438-9d6e-12fac8aa9d68</t>
+  </si>
+  <si>
+    <t>Vongdeuan jewelry shop</t>
+  </si>
+  <si>
+    <t>2026-03-28</t>
+  </si>
+  <si>
+    <t>/uploads/1774674648047-PHOTO-2026-03-28-12-04-41.jpg</t>
+  </si>
+  <si>
+    <t>2026-03-28T05:10:48.435Z</t>
+  </si>
+  <si>
+    <t>87bdc6f2-ff12-49e8-98bc-cd37f5bf28b5</t>
+  </si>
+  <si>
+    <t>Bonus for employees</t>
+  </si>
+  <si>
+    <t>/uploads/1774678317982-PHOTO-2026-03-28-13-02-42.jpg</t>
+  </si>
+  <si>
+    <t>2026-03-28T06:11:59.509Z</t>
+  </si>
+  <si>
+    <t>2123c29b-6727-49b4-bfbd-51b830d0ef24</t>
+  </si>
+  <si>
+    <t>Advertising services facebook</t>
+  </si>
+  <si>
+    <t>/uploads/1774680809823-PHOTO-2026-03-28-13-46-55.jpg</t>
+  </si>
+  <si>
+    <t>2026-03-28T06:53:29.824Z</t>
+  </si>
+  <si>
+    <t>10c6c562-f371-4896-a83c-4d862ac68e62</t>
+  </si>
+  <si>
+    <t>Coffee cup plate set</t>
+  </si>
+  <si>
+    <t>2026-03-31</t>
+  </si>
+  <si>
+    <t>/uploads/1774950262906-WhatsApp_Image_2026-03-31_at_1_30_23___PM.jpeg</t>
+  </si>
+  <si>
+    <t>2026-03-31T09:44:22.909Z</t>
+  </si>
+  <si>
+    <t>a393b10c-5fcd-4705-b2d0-a928f09b45c4</t>
+  </si>
+  <si>
+    <t>/uploads/1774950324096-WhatsApp_Image_2026-03-31_at_1_30_23___PM.jpeg</t>
+  </si>
+  <si>
+    <t>2026-03-31T09:45:25.983Z</t>
+  </si>
+  <si>
+    <t>e131225a-5735-4334-a4ec-73658325bb5a</t>
+  </si>
+  <si>
+    <t>Umbrella</t>
+  </si>
+  <si>
+    <t>2026-04-01</t>
+  </si>
+  <si>
+    <t>/uploads/1775041032324-PHOTO-2026-04-01-16-30-04.jpg</t>
+  </si>
+  <si>
+    <t>2026-04-01T10:57:15.775Z</t>
+  </si>
+  <si>
+    <t>357a23e6-2ce6-4af6-8b49-19a8b455fe5c</t>
+  </si>
+  <si>
+    <t>Examples of cap</t>
+  </si>
+  <si>
+    <t>/uploads/1775041391869-PHOTO-2026-04-01-16-30-45.jpg</t>
+  </si>
+  <si>
+    <t>2026-04-01T11:03:14.709Z</t>
+  </si>
+  <si>
+    <t>76148e58-8ca5-4173-b49b-d2df9d6b0ac1</t>
+  </si>
+  <si>
+    <t>Employee allowance</t>
+  </si>
+  <si>
+    <t>2026-04-02</t>
+  </si>
+  <si>
+    <t>/uploads/1775109138953-98744e7c-0e52-4f91-93e6-a52faf84a001.jpeg</t>
+  </si>
+  <si>
+    <t>2026-04-02T05:52:21.166Z</t>
+  </si>
+  <si>
+    <t>d6f29352-b043-4fa8-bfa1-f103e29db78b</t>
+  </si>
+  <si>
+    <t>Car Front windshield Sunshade</t>
+  </si>
+  <si>
+    <t>2026-04-04</t>
+  </si>
+  <si>
+    <t>/uploads/1775273246551-PHOTO-2026-04-03-10-21-39.jpg</t>
+  </si>
+  <si>
+    <t>2026-04-04T03:27:27.892Z</t>
+  </si>
+  <si>
+    <t>ba38326f-af10-470f-810d-3efa52fc3bed</t>
+  </si>
+  <si>
+    <t>Laser machine</t>
+  </si>
+  <si>
+    <t>/uploads/1775273603639-PHOTO-2026-04-04-09-09-46.jpg</t>
+  </si>
+  <si>
+    <t>2026-04-04T03:33:23.640Z</t>
+  </si>
+  <si>
+    <t>8d182ce3-5863-4685-90d5-03ba4a5d18f0</t>
+  </si>
+  <si>
+    <t>Document envelope</t>
+  </si>
+  <si>
+    <t>2026-04-06</t>
+  </si>
+  <si>
+    <t>/uploads/1775454024177-WhatsApp_Image_2026-04-05_at_10_02_47___AM.jpeg</t>
+  </si>
+  <si>
+    <t>2026-04-06T05:40:24.814Z</t>
+  </si>
+  <si>
+    <t>94e2cca7-5bb9-4827-9360-1de0c0ce2161</t>
+  </si>
+  <si>
+    <t>/uploads/1775454074667-WhatsApp_Image_2026-04-05_at_10_02_48___AM.jpeg</t>
+  </si>
+  <si>
+    <t>2026-04-06T05:41:15.212Z</t>
+  </si>
+  <si>
+    <t>d22aac6a-bc72-4796-91fb-ac873dd82a2c</t>
+  </si>
+  <si>
+    <t>Example of cap</t>
+  </si>
+  <si>
+    <t>/uploads/1775455240252-WhatsApp_Image_2026-04-05_at_10_02_48___AM__1_.jpeg</t>
+  </si>
+  <si>
+    <t>2026-04-06T06:00:41.398Z</t>
+  </si>
+  <si>
+    <t>b69a2609-5cff-41cb-873c-f857b9c5c649</t>
+  </si>
+  <si>
+    <t>Mini phone shop shipping costs</t>
+  </si>
+  <si>
+    <t>/uploads/1775455555662-WhatsApp_Image_2026-04-06_at_9_16_32___AM.jpeg</t>
+  </si>
+  <si>
+    <t>2026-04-06T06:05:56.212Z</t>
+  </si>
+  <si>
+    <t>2026-04-06T06:05:56.213Z</t>
+  </si>
+  <si>
+    <t>aa3410b4-3ef5-45ed-b25d-9310aca4a5a3</t>
+  </si>
+  <si>
+    <t>Vongduean shop shipping costs</t>
+  </si>
+  <si>
+    <t>/uploads/1775455722466-WhatsApp_Image_2026-04-06_at_9_16_33___AM.jpeg</t>
+  </si>
+  <si>
+    <t>2026-04-06T06:08:43.430Z</t>
+  </si>
+  <si>
+    <t>205a2445-dd20-4d60-9ed0-cca7cb37a2a9</t>
+  </si>
+  <si>
+    <t>Mug 30%</t>
+  </si>
+  <si>
+    <t>/uploads/1775456264222-a50488f6-774e-48ac-88d3-b2eb95734448_052BAAE7-4466-4148-BC74-EC28713C843E.jpeg</t>
+  </si>
+  <si>
+    <t>2026-04-06T06:17:44.488Z</t>
+  </si>
+  <si>
+    <t>3b88b19f-9178-4167-952e-770d9899d926</t>
+  </si>
+  <si>
+    <t>Laser machine shipping costs</t>
+  </si>
+  <si>
+    <t>/uploads/1775456350157-d89d3fd6-aec6-41b6-b931-1ead9b4da5fc_48BED14F-649A-4724-BCDE-B4856238ABA9.jpeg</t>
+  </si>
+  <si>
+    <t>2026-04-06T06:19:12.608Z</t>
+  </si>
+  <si>
+    <t>333e3881-808f-4cc5-a1b9-c25e4097aa69</t>
+  </si>
+  <si>
+    <t>Tourism Malaysia shipping costs</t>
+  </si>
+  <si>
+    <t>/uploads/1775468248344-WhatsApp_Image_2026-04-06_at_9_16_33___AM__1_.jpeg</t>
+  </si>
+  <si>
+    <t>2026-04-06T09:37:29.564Z</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -589,14 +1235,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L3"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:L8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="12" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" s="1" customFormat="1" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -634,7 +1280,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -672,7 +1318,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>22</v>
       </c>
@@ -710,21 +1356,211 @@
         <v>31</v>
       </c>
     </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E4" t="s">
+        <v>63</v>
+      </c>
+      <c r="F4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G4" t="s">
+        <v>65</v>
+      </c>
+      <c r="H4" t="s">
+        <v>66</v>
+      </c>
+      <c r="I4" t="s">
+        <v>67</v>
+      </c>
+      <c r="J4" t="s">
+        <v>68</v>
+      </c>
+      <c r="K4" t="s">
+        <v>69</v>
+      </c>
+      <c r="L4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5" t="s">
+        <v>71</v>
+      </c>
+      <c r="D5" t="s">
+        <v>72</v>
+      </c>
+      <c r="E5" t="s">
+        <v>73</v>
+      </c>
+      <c r="F5" t="s">
+        <v>64</v>
+      </c>
+      <c r="G5" t="s">
+        <v>65</v>
+      </c>
+      <c r="H5" t="s">
+        <v>66</v>
+      </c>
+      <c r="I5" t="s">
+        <v>74</v>
+      </c>
+      <c r="J5" t="s">
+        <v>75</v>
+      </c>
+      <c r="K5" t="s">
+        <v>76</v>
+      </c>
+      <c r="L5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>77</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>78</v>
+      </c>
+      <c r="D6" t="s">
+        <v>79</v>
+      </c>
+      <c r="E6" t="s">
+        <v>80</v>
+      </c>
+      <c r="F6" t="s">
+        <v>64</v>
+      </c>
+      <c r="G6" t="s">
+        <v>65</v>
+      </c>
+      <c r="H6" t="s">
+        <v>81</v>
+      </c>
+      <c r="I6" t="s">
+        <v>82</v>
+      </c>
+      <c r="J6" t="s">
+        <v>83</v>
+      </c>
+      <c r="K6" t="s">
+        <v>84</v>
+      </c>
+      <c r="L6" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>85</v>
+      </c>
+      <c r="B7">
+        <v>6</v>
+      </c>
+      <c r="C7" t="s">
+        <v>86</v>
+      </c>
+      <c r="D7" t="s">
+        <v>87</v>
+      </c>
+      <c r="E7" t="s">
+        <v>88</v>
+      </c>
+      <c r="F7" t="s">
+        <v>64</v>
+      </c>
+      <c r="G7" t="s">
+        <v>65</v>
+      </c>
+      <c r="H7" t="s">
+        <v>89</v>
+      </c>
+      <c r="I7" t="s">
+        <v>90</v>
+      </c>
+      <c r="J7" t="s">
+        <v>91</v>
+      </c>
+      <c r="K7" t="s">
+        <v>92</v>
+      </c>
+      <c r="L7" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>93</v>
+      </c>
+      <c r="B8">
+        <v>7</v>
+      </c>
+      <c r="C8" t="s">
+        <v>94</v>
+      </c>
+      <c r="D8" t="s">
+        <v>95</v>
+      </c>
+      <c r="E8" t="s">
+        <v>96</v>
+      </c>
+      <c r="F8" t="s">
+        <v>64</v>
+      </c>
+      <c r="G8" t="s">
+        <v>65</v>
+      </c>
+      <c r="H8" t="s">
+        <v>89</v>
+      </c>
+      <c r="I8" t="s">
+        <v>97</v>
+      </c>
+      <c r="J8" t="s">
+        <v>98</v>
+      </c>
+      <c r="K8" t="s">
+        <v>99</v>
+      </c>
+      <c r="L8" t="s">
+        <v>99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L5"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:L40"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="12" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" s="1" customFormat="1" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -762,7 +1598,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>39</v>
       </c>
@@ -800,7 +1636,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>45</v>
       </c>
@@ -838,7 +1674,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>51</v>
       </c>
@@ -876,7 +1712,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>55</v>
       </c>
@@ -914,8 +1750,1338 @@
         <v>59</v>
       </c>
     </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>100</v>
+      </c>
+      <c r="B6">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" t="s">
+        <v>101</v>
+      </c>
+      <c r="G6" t="s">
+        <v>42</v>
+      </c>
+      <c r="H6">
+        <v>50000</v>
+      </c>
+      <c r="I6" t="s">
+        <v>102</v>
+      </c>
+      <c r="J6" t="s">
+        <v>103</v>
+      </c>
+      <c r="K6" t="s">
+        <v>104</v>
+      </c>
+      <c r="L6" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>105</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" t="s">
+        <v>106</v>
+      </c>
+      <c r="E7" t="s">
+        <v>107</v>
+      </c>
+      <c r="F7" t="s">
+        <v>108</v>
+      </c>
+      <c r="G7" t="s">
+        <v>42</v>
+      </c>
+      <c r="H7">
+        <v>5204176</v>
+      </c>
+      <c r="I7" t="s">
+        <v>102</v>
+      </c>
+      <c r="J7" t="s">
+        <v>109</v>
+      </c>
+      <c r="K7" t="s">
+        <v>110</v>
+      </c>
+      <c r="L7" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>111</v>
+      </c>
+      <c r="B8">
+        <v>5</v>
+      </c>
+      <c r="C8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" t="s">
+        <v>40</v>
+      </c>
+      <c r="E8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" t="s">
+        <v>108</v>
+      </c>
+      <c r="G8" t="s">
+        <v>42</v>
+      </c>
+      <c r="H8">
+        <v>4489700</v>
+      </c>
+      <c r="I8" t="s">
+        <v>102</v>
+      </c>
+      <c r="J8" t="s">
+        <v>112</v>
+      </c>
+      <c r="K8" t="s">
+        <v>113</v>
+      </c>
+      <c r="L8" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>114</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" t="s">
+        <v>70</v>
+      </c>
+      <c r="D9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E9" t="s">
+        <v>115</v>
+      </c>
+      <c r="F9" t="s">
+        <v>115</v>
+      </c>
+      <c r="G9" t="s">
+        <v>42</v>
+      </c>
+      <c r="H9">
+        <v>969000</v>
+      </c>
+      <c r="I9" t="s">
+        <v>102</v>
+      </c>
+      <c r="J9" t="s">
+        <v>116</v>
+      </c>
+      <c r="K9" t="s">
+        <v>117</v>
+      </c>
+      <c r="L9" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>118</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" t="s">
+        <v>106</v>
+      </c>
+      <c r="E10" t="s">
+        <v>107</v>
+      </c>
+      <c r="F10" t="s">
+        <v>119</v>
+      </c>
+      <c r="G10" t="s">
+        <v>42</v>
+      </c>
+      <c r="H10">
+        <v>4657660</v>
+      </c>
+      <c r="I10" t="s">
+        <v>102</v>
+      </c>
+      <c r="J10" t="s">
+        <v>120</v>
+      </c>
+      <c r="K10" t="s">
+        <v>121</v>
+      </c>
+      <c r="L10" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>122</v>
+      </c>
+      <c r="B11">
+        <v>1</v>
+      </c>
+      <c r="C11" t="s">
+        <v>60</v>
+      </c>
+      <c r="D11" t="s">
+        <v>106</v>
+      </c>
+      <c r="E11" t="s">
+        <v>107</v>
+      </c>
+      <c r="F11" t="s">
+        <v>108</v>
+      </c>
+      <c r="G11" t="s">
+        <v>42</v>
+      </c>
+      <c r="H11">
+        <v>9496200</v>
+      </c>
+      <c r="I11" t="s">
+        <v>123</v>
+      </c>
+      <c r="J11" t="s">
+        <v>124</v>
+      </c>
+      <c r="K11" t="s">
+        <v>125</v>
+      </c>
+      <c r="L11" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>126</v>
+      </c>
+      <c r="B12">
+        <v>2</v>
+      </c>
+      <c r="C12" t="s">
+        <v>60</v>
+      </c>
+      <c r="D12" t="s">
+        <v>106</v>
+      </c>
+      <c r="E12" t="s">
+        <v>107</v>
+      </c>
+      <c r="F12" t="s">
+        <v>127</v>
+      </c>
+      <c r="G12" t="s">
+        <v>42</v>
+      </c>
+      <c r="H12">
+        <v>187340</v>
+      </c>
+      <c r="I12" t="s">
+        <v>123</v>
+      </c>
+      <c r="J12" t="s">
+        <v>128</v>
+      </c>
+      <c r="K12" t="s">
+        <v>129</v>
+      </c>
+      <c r="L12" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>130</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>60</v>
+      </c>
+      <c r="D13" t="s">
+        <v>106</v>
+      </c>
+      <c r="E13" t="s">
+        <v>107</v>
+      </c>
+      <c r="F13" t="s">
+        <v>127</v>
+      </c>
+      <c r="G13" t="s">
+        <v>42</v>
+      </c>
+      <c r="H13">
+        <v>6460000</v>
+      </c>
+      <c r="I13" t="s">
+        <v>123</v>
+      </c>
+      <c r="J13" t="s">
+        <v>131</v>
+      </c>
+      <c r="K13" t="s">
+        <v>132</v>
+      </c>
+      <c r="L13" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>133</v>
+      </c>
+      <c r="B14">
+        <v>6</v>
+      </c>
+      <c r="C14" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" t="s">
+        <v>46</v>
+      </c>
+      <c r="E14" t="s">
+        <v>134</v>
+      </c>
+      <c r="F14" t="s">
+        <v>134</v>
+      </c>
+      <c r="G14" t="s">
+        <v>42</v>
+      </c>
+      <c r="H14">
+        <v>5250000</v>
+      </c>
+      <c r="I14" t="s">
+        <v>123</v>
+      </c>
+      <c r="J14" t="s">
+        <v>135</v>
+      </c>
+      <c r="K14" t="s">
+        <v>136</v>
+      </c>
+      <c r="L14" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>137</v>
+      </c>
+      <c r="B15">
+        <v>7</v>
+      </c>
+      <c r="C15" t="s">
+        <v>12</v>
+      </c>
+      <c r="D15" t="s">
+        <v>40</v>
+      </c>
+      <c r="E15" t="s">
+        <v>15</v>
+      </c>
+      <c r="F15" t="s">
+        <v>138</v>
+      </c>
+      <c r="G15" t="s">
+        <v>42</v>
+      </c>
+      <c r="H15">
+        <v>108040</v>
+      </c>
+      <c r="I15" t="s">
+        <v>139</v>
+      </c>
+      <c r="J15" t="s">
+        <v>140</v>
+      </c>
+      <c r="K15" t="s">
+        <v>141</v>
+      </c>
+      <c r="L15" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>142</v>
+      </c>
+      <c r="B16">
+        <v>2</v>
+      </c>
+      <c r="C16" t="s">
+        <v>70</v>
+      </c>
+      <c r="D16" t="s">
+        <v>40</v>
+      </c>
+      <c r="E16" t="s">
+        <v>115</v>
+      </c>
+      <c r="F16" t="s">
+        <v>115</v>
+      </c>
+      <c r="G16" t="s">
+        <v>42</v>
+      </c>
+      <c r="H16">
+        <v>32300</v>
+      </c>
+      <c r="I16" t="s">
+        <v>143</v>
+      </c>
+      <c r="J16" t="s">
+        <v>144</v>
+      </c>
+      <c r="K16" t="s">
+        <v>145</v>
+      </c>
+      <c r="L16" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>146</v>
+      </c>
+      <c r="B17">
+        <v>8</v>
+      </c>
+      <c r="C17" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" t="s">
+        <v>40</v>
+      </c>
+      <c r="E17" t="s">
+        <v>147</v>
+      </c>
+      <c r="F17" t="s">
+        <v>147</v>
+      </c>
+      <c r="G17" t="s">
+        <v>42</v>
+      </c>
+      <c r="H17">
+        <v>590346</v>
+      </c>
+      <c r="I17" t="s">
+        <v>148</v>
+      </c>
+      <c r="J17" t="s">
+        <v>149</v>
+      </c>
+      <c r="K17" t="s">
+        <v>150</v>
+      </c>
+      <c r="L17" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>151</v>
+      </c>
+      <c r="B18">
+        <v>9</v>
+      </c>
+      <c r="C18" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" t="s">
+        <v>40</v>
+      </c>
+      <c r="E18" t="s">
+        <v>15</v>
+      </c>
+      <c r="F18" t="s">
+        <v>56</v>
+      </c>
+      <c r="G18" t="s">
+        <v>42</v>
+      </c>
+      <c r="H18">
+        <v>75000</v>
+      </c>
+      <c r="I18" t="s">
+        <v>152</v>
+      </c>
+      <c r="J18" t="s">
+        <v>153</v>
+      </c>
+      <c r="K18" t="s">
+        <v>154</v>
+      </c>
+      <c r="L18" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>155</v>
+      </c>
+      <c r="B19">
+        <v>10</v>
+      </c>
+      <c r="C19" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" t="s">
+        <v>40</v>
+      </c>
+      <c r="E19" t="s">
+        <v>15</v>
+      </c>
+      <c r="F19" t="s">
+        <v>156</v>
+      </c>
+      <c r="G19" t="s">
+        <v>42</v>
+      </c>
+      <c r="H19">
+        <v>1296000</v>
+      </c>
+      <c r="I19" t="s">
+        <v>157</v>
+      </c>
+      <c r="J19" t="s">
+        <v>158</v>
+      </c>
+      <c r="K19" t="s">
+        <v>159</v>
+      </c>
+      <c r="L19" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>160</v>
+      </c>
+      <c r="B20">
+        <v>1</v>
+      </c>
+      <c r="C20" t="s">
+        <v>77</v>
+      </c>
+      <c r="D20" t="s">
+        <v>46</v>
+      </c>
+      <c r="E20" t="s">
+        <v>47</v>
+      </c>
+      <c r="F20" t="s">
+        <v>80</v>
+      </c>
+      <c r="G20" t="s">
+        <v>42</v>
+      </c>
+      <c r="H20">
+        <v>8490000</v>
+      </c>
+      <c r="I20" t="s">
+        <v>157</v>
+      </c>
+      <c r="J20" t="s">
+        <v>161</v>
+      </c>
+      <c r="K20" t="s">
+        <v>162</v>
+      </c>
+      <c r="L20" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>163</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21" t="s">
+        <v>77</v>
+      </c>
+      <c r="D21" t="s">
+        <v>106</v>
+      </c>
+      <c r="E21" t="s">
+        <v>47</v>
+      </c>
+      <c r="F21" t="s">
+        <v>164</v>
+      </c>
+      <c r="G21" t="s">
+        <v>42</v>
+      </c>
+      <c r="H21">
+        <v>1889000</v>
+      </c>
+      <c r="I21" t="s">
+        <v>157</v>
+      </c>
+      <c r="J21" t="s">
+        <v>165</v>
+      </c>
+      <c r="K21" t="s">
+        <v>166</v>
+      </c>
+      <c r="L21" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>167</v>
+      </c>
+      <c r="B22">
+        <v>3</v>
+      </c>
+      <c r="C22" t="s">
+        <v>77</v>
+      </c>
+      <c r="D22" t="s">
+        <v>106</v>
+      </c>
+      <c r="E22" t="s">
+        <v>47</v>
+      </c>
+      <c r="F22" t="s">
+        <v>168</v>
+      </c>
+      <c r="G22" t="s">
+        <v>42</v>
+      </c>
+      <c r="H22">
+        <v>1312000</v>
+      </c>
+      <c r="I22" t="s">
+        <v>157</v>
+      </c>
+      <c r="J22" t="s">
+        <v>169</v>
+      </c>
+      <c r="K22" t="s">
+        <v>170</v>
+      </c>
+      <c r="L22" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>171</v>
+      </c>
+      <c r="B23">
+        <v>11</v>
+      </c>
+      <c r="C23" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23" t="s">
+        <v>46</v>
+      </c>
+      <c r="E23" t="s">
+        <v>108</v>
+      </c>
+      <c r="F23" t="s">
+        <v>172</v>
+      </c>
+      <c r="G23" t="s">
+        <v>42</v>
+      </c>
+      <c r="H23">
+        <v>29756000</v>
+      </c>
+      <c r="I23" t="s">
+        <v>173</v>
+      </c>
+      <c r="J23" t="s">
+        <v>174</v>
+      </c>
+      <c r="K23" t="s">
+        <v>175</v>
+      </c>
+      <c r="L23" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>176</v>
+      </c>
+      <c r="B24">
+        <v>12</v>
+      </c>
+      <c r="C24" t="s">
+        <v>12</v>
+      </c>
+      <c r="D24" t="s">
+        <v>40</v>
+      </c>
+      <c r="E24" t="s">
+        <v>15</v>
+      </c>
+      <c r="F24" t="s">
+        <v>177</v>
+      </c>
+      <c r="G24" t="s">
+        <v>42</v>
+      </c>
+      <c r="H24">
+        <v>32396000</v>
+      </c>
+      <c r="I24" t="s">
+        <v>173</v>
+      </c>
+      <c r="J24" t="s">
+        <v>178</v>
+      </c>
+      <c r="K24" t="s">
+        <v>179</v>
+      </c>
+      <c r="L24" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>180</v>
+      </c>
+      <c r="B25">
+        <v>13</v>
+      </c>
+      <c r="C25" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25" t="s">
+        <v>40</v>
+      </c>
+      <c r="E25" t="s">
+        <v>15</v>
+      </c>
+      <c r="F25" t="s">
+        <v>181</v>
+      </c>
+      <c r="G25" t="s">
+        <v>42</v>
+      </c>
+      <c r="H25">
+        <v>750150</v>
+      </c>
+      <c r="I25" t="s">
+        <v>173</v>
+      </c>
+      <c r="J25" t="s">
+        <v>182</v>
+      </c>
+      <c r="K25" t="s">
+        <v>183</v>
+      </c>
+      <c r="L25" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>184</v>
+      </c>
+      <c r="B26">
+        <v>4</v>
+      </c>
+      <c r="C26" t="s">
+        <v>77</v>
+      </c>
+      <c r="D26" t="s">
+        <v>106</v>
+      </c>
+      <c r="E26" t="s">
+        <v>107</v>
+      </c>
+      <c r="F26" t="s">
+        <v>185</v>
+      </c>
+      <c r="G26" t="s">
+        <v>42</v>
+      </c>
+      <c r="H26">
+        <v>9925000</v>
+      </c>
+      <c r="I26" t="s">
+        <v>186</v>
+      </c>
+      <c r="J26" t="s">
+        <v>187</v>
+      </c>
+      <c r="K26" t="s">
+        <v>188</v>
+      </c>
+      <c r="L26" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>189</v>
+      </c>
+      <c r="B27">
+        <v>5</v>
+      </c>
+      <c r="C27" t="s">
+        <v>77</v>
+      </c>
+      <c r="D27" t="s">
+        <v>46</v>
+      </c>
+      <c r="E27" t="s">
+        <v>107</v>
+      </c>
+      <c r="F27" t="s">
+        <v>185</v>
+      </c>
+      <c r="G27" t="s">
+        <v>42</v>
+      </c>
+      <c r="H27">
+        <v>790000</v>
+      </c>
+      <c r="I27" t="s">
+        <v>186</v>
+      </c>
+      <c r="J27" t="s">
+        <v>190</v>
+      </c>
+      <c r="K27" t="s">
+        <v>191</v>
+      </c>
+      <c r="L27" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>192</v>
+      </c>
+      <c r="B28">
+        <v>4</v>
+      </c>
+      <c r="C28" t="s">
+        <v>22</v>
+      </c>
+      <c r="D28" t="s">
+        <v>40</v>
+      </c>
+      <c r="E28" t="s">
+        <v>107</v>
+      </c>
+      <c r="F28" t="s">
+        <v>193</v>
+      </c>
+      <c r="G28" t="s">
+        <v>42</v>
+      </c>
+      <c r="H28">
+        <v>7672000</v>
+      </c>
+      <c r="I28" t="s">
+        <v>194</v>
+      </c>
+      <c r="J28" t="s">
+        <v>195</v>
+      </c>
+      <c r="K28" t="s">
+        <v>196</v>
+      </c>
+      <c r="L28" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>197</v>
+      </c>
+      <c r="B29">
+        <v>3</v>
+      </c>
+      <c r="C29" t="s">
+        <v>70</v>
+      </c>
+      <c r="D29" t="s">
+        <v>40</v>
+      </c>
+      <c r="E29" t="s">
+        <v>15</v>
+      </c>
+      <c r="F29" t="s">
+        <v>198</v>
+      </c>
+      <c r="G29" t="s">
+        <v>42</v>
+      </c>
+      <c r="H29">
+        <v>264000</v>
+      </c>
+      <c r="I29" t="s">
+        <v>194</v>
+      </c>
+      <c r="J29" t="s">
+        <v>199</v>
+      </c>
+      <c r="K29" t="s">
+        <v>200</v>
+      </c>
+      <c r="L29" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>201</v>
+      </c>
+      <c r="B30">
+        <v>4</v>
+      </c>
+      <c r="C30" t="s">
+        <v>70</v>
+      </c>
+      <c r="D30" t="s">
+        <v>40</v>
+      </c>
+      <c r="E30" t="s">
+        <v>15</v>
+      </c>
+      <c r="F30" t="s">
+        <v>202</v>
+      </c>
+      <c r="G30" t="s">
+        <v>42</v>
+      </c>
+      <c r="H30">
+        <v>1168000</v>
+      </c>
+      <c r="I30" t="s">
+        <v>203</v>
+      </c>
+      <c r="J30" t="s">
+        <v>204</v>
+      </c>
+      <c r="K30" t="s">
+        <v>205</v>
+      </c>
+      <c r="L30" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>206</v>
+      </c>
+      <c r="B31">
+        <v>5</v>
+      </c>
+      <c r="C31" t="s">
+        <v>70</v>
+      </c>
+      <c r="D31" t="s">
+        <v>106</v>
+      </c>
+      <c r="E31" t="s">
+        <v>107</v>
+      </c>
+      <c r="F31" t="s">
+        <v>207</v>
+      </c>
+      <c r="G31" t="s">
+        <v>42</v>
+      </c>
+      <c r="H31">
+        <v>25157000</v>
+      </c>
+      <c r="I31" t="s">
+        <v>208</v>
+      </c>
+      <c r="J31" t="s">
+        <v>209</v>
+      </c>
+      <c r="K31" t="s">
+        <v>210</v>
+      </c>
+      <c r="L31" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>211</v>
+      </c>
+      <c r="B32">
+        <v>14</v>
+      </c>
+      <c r="C32" t="s">
+        <v>12</v>
+      </c>
+      <c r="D32" t="s">
+        <v>40</v>
+      </c>
+      <c r="E32" t="s">
+        <v>15</v>
+      </c>
+      <c r="F32" t="s">
+        <v>212</v>
+      </c>
+      <c r="G32" t="s">
+        <v>42</v>
+      </c>
+      <c r="H32">
+        <v>11470200</v>
+      </c>
+      <c r="I32" t="s">
+        <v>208</v>
+      </c>
+      <c r="J32" t="s">
+        <v>213</v>
+      </c>
+      <c r="K32" t="s">
+        <v>214</v>
+      </c>
+      <c r="L32" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>215</v>
+      </c>
+      <c r="B33">
+        <v>5</v>
+      </c>
+      <c r="C33" t="s">
+        <v>22</v>
+      </c>
+      <c r="D33" t="s">
+        <v>106</v>
+      </c>
+      <c r="E33" t="s">
+        <v>107</v>
+      </c>
+      <c r="F33" t="s">
+        <v>216</v>
+      </c>
+      <c r="G33" t="s">
+        <v>42</v>
+      </c>
+      <c r="H33">
+        <v>7036000</v>
+      </c>
+      <c r="I33" t="s">
+        <v>217</v>
+      </c>
+      <c r="J33" t="s">
+        <v>218</v>
+      </c>
+      <c r="K33" t="s">
+        <v>219</v>
+      </c>
+      <c r="L33" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>220</v>
+      </c>
+      <c r="B34">
+        <v>6</v>
+      </c>
+      <c r="C34" t="s">
+        <v>22</v>
+      </c>
+      <c r="D34" t="s">
+        <v>106</v>
+      </c>
+      <c r="E34" t="s">
+        <v>107</v>
+      </c>
+      <c r="F34" t="s">
+        <v>216</v>
+      </c>
+      <c r="G34" t="s">
+        <v>42</v>
+      </c>
+      <c r="H34">
+        <v>5592000</v>
+      </c>
+      <c r="I34" t="s">
+        <v>217</v>
+      </c>
+      <c r="J34" t="s">
+        <v>221</v>
+      </c>
+      <c r="K34" t="s">
+        <v>222</v>
+      </c>
+      <c r="L34" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>223</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35" t="s">
+        <v>85</v>
+      </c>
+      <c r="D35" t="s">
+        <v>106</v>
+      </c>
+      <c r="E35" t="s">
+        <v>115</v>
+      </c>
+      <c r="F35" t="s">
+        <v>224</v>
+      </c>
+      <c r="G35" t="s">
+        <v>42</v>
+      </c>
+      <c r="H35">
+        <v>1968000</v>
+      </c>
+      <c r="I35" t="s">
+        <v>217</v>
+      </c>
+      <c r="J35" t="s">
+        <v>225</v>
+      </c>
+      <c r="K35" t="s">
+        <v>226</v>
+      </c>
+      <c r="L35" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>227</v>
+      </c>
+      <c r="B36">
+        <v>15</v>
+      </c>
+      <c r="C36" t="s">
+        <v>12</v>
+      </c>
+      <c r="D36" t="s">
+        <v>40</v>
+      </c>
+      <c r="E36" t="s">
+        <v>15</v>
+      </c>
+      <c r="F36" t="s">
+        <v>228</v>
+      </c>
+      <c r="G36" t="s">
+        <v>42</v>
+      </c>
+      <c r="H36">
+        <v>410000</v>
+      </c>
+      <c r="I36" t="s">
+        <v>217</v>
+      </c>
+      <c r="J36" t="s">
+        <v>229</v>
+      </c>
+      <c r="K36" t="s">
+        <v>230</v>
+      </c>
+      <c r="L36" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>232</v>
+      </c>
+      <c r="B37">
+        <v>16</v>
+      </c>
+      <c r="C37" t="s">
+        <v>12</v>
+      </c>
+      <c r="D37" t="s">
+        <v>40</v>
+      </c>
+      <c r="E37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F37" t="s">
+        <v>233</v>
+      </c>
+      <c r="G37" t="s">
+        <v>42</v>
+      </c>
+      <c r="H37">
+        <v>940000</v>
+      </c>
+      <c r="I37" t="s">
+        <v>217</v>
+      </c>
+      <c r="J37" t="s">
+        <v>234</v>
+      </c>
+      <c r="K37" t="s">
+        <v>235</v>
+      </c>
+      <c r="L37" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>236</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" t="s">
+        <v>93</v>
+      </c>
+      <c r="D38" t="s">
+        <v>46</v>
+      </c>
+      <c r="E38" t="s">
+        <v>47</v>
+      </c>
+      <c r="F38" t="s">
+        <v>237</v>
+      </c>
+      <c r="G38" t="s">
+        <v>42</v>
+      </c>
+      <c r="H38">
+        <v>2000000</v>
+      </c>
+      <c r="I38" t="s">
+        <v>217</v>
+      </c>
+      <c r="J38" t="s">
+        <v>238</v>
+      </c>
+      <c r="K38" t="s">
+        <v>239</v>
+      </c>
+      <c r="L38" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>240</v>
+      </c>
+      <c r="B39">
+        <v>18</v>
+      </c>
+      <c r="C39" t="s">
+        <v>12</v>
+      </c>
+      <c r="D39" t="s">
+        <v>40</v>
+      </c>
+      <c r="E39" t="s">
+        <v>15</v>
+      </c>
+      <c r="F39" t="s">
+        <v>241</v>
+      </c>
+      <c r="G39" t="s">
+        <v>42</v>
+      </c>
+      <c r="H39">
+        <v>137000</v>
+      </c>
+      <c r="I39" t="s">
+        <v>217</v>
+      </c>
+      <c r="J39" t="s">
+        <v>242</v>
+      </c>
+      <c r="K39" t="s">
+        <v>243</v>
+      </c>
+      <c r="L39" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>244</v>
+      </c>
+      <c r="B40">
+        <v>4</v>
+      </c>
+      <c r="C40" t="s">
+        <v>60</v>
+      </c>
+      <c r="D40" t="s">
+        <v>40</v>
+      </c>
+      <c r="E40" t="s">
+        <v>15</v>
+      </c>
+      <c r="F40" t="s">
+        <v>245</v>
+      </c>
+      <c r="G40" t="s">
+        <v>42</v>
+      </c>
+      <c r="H40">
+        <v>1442000</v>
+      </c>
+      <c r="I40" t="s">
+        <v>217</v>
+      </c>
+      <c r="J40" t="s">
+        <v>246</v>
+      </c>
+      <c r="K40" t="s">
+        <v>247</v>
+      </c>
+      <c r="L40" t="s">
+        <v>247</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>